<commit_message>
chore: rename bagisto/ to store/
Directory name is arbitrary to PHP/Composer; only docs, .gitignore
and the Dockerfile overlay pattern referenced it. Server + suite
verified from the new path.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.original.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.original.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -551,44 +551,52 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -688,34 +696,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -861,148 +869,148 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <f aca="false">COUNTA('3-Day Plan'!B5:B21)</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="4" t="n">
         <f aca="false">COUNTIF('3-Day Plan'!E5:E21,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <f aca="false">COUNTIF('3-Day Plan'!E5:E21,"In progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <f aca="false">COUNTIF('3-Day Plan'!E5:E21,"Cut")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="n">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="n">
         <f aca="false">COUNTIF('3-Day Plan'!E5:E21,"Not started")</f>
         <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <f aca="false">IF(B4-B7=0,0,B5/(B4-B7))</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="4" t="n">
         <f aca="false">COUNTIF('Gap List'!F5:F21,"Yes")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="4" t="n">
         <f aca="false">COUNTA('Gap List'!B5:B21)</f>
         <v>17</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="4" t="n">
         <f aca="false">COUNTIF('Gap List'!D5:D21,"Built-in*")</f>
         <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="4" t="n">
         <f aca="false">COUNTIF('Gap List'!D5:D21,"Config*")</f>
         <v>5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="4" t="n">
         <f aca="false">COUNTIF('Gap List'!D5:D21,"Small code change*")</f>
         <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="4" t="n">
         <f aca="false">COUNTIF('Gap List'!D5:D21,"Custom code*")</f>
         <v>2</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1023,415 +1031,422 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>19</v>
       </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="3" t="s">
+      <c r="F5" s="10"/>
+      <c r="G5" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="3" t="s">
+      <c r="F6" s="10"/>
+      <c r="G6" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="10"/>
+      <c r="G7" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="3" t="s">
+      <c r="F8" s="10"/>
+      <c r="G8" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="3" t="s">
+      <c r="F9" s="10"/>
+      <c r="G9" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="3" t="s">
+      <c r="F10" s="10"/>
+      <c r="G10" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="3" t="s">
+      <c r="F11" s="10"/>
+      <c r="G11" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="3" t="s">
+      <c r="F12" s="10"/>
+      <c r="G12" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="3" t="s">
+      <c r="F13" s="10"/>
+      <c r="G13" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="3" t="s">
+      <c r="F14" s="10"/>
+      <c r="G14" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="3" t="s">
+      <c r="F15" s="10"/>
+      <c r="G15" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="3" t="s">
+      <c r="F16" s="10"/>
+      <c r="G16" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="3" t="s">
+      <c r="F17" s="10"/>
+      <c r="G17" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="3" t="s">
+      <c r="F18" s="10"/>
+      <c r="G18" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="3" t="s">
+      <c r="F19" s="10"/>
+      <c r="G19" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="3" t="s">
+      <c r="F20" s="10"/>
+      <c r="G20" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="3" t="s">
+      <c r="F21" s="10"/>
+      <c r="G21" s="4" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="1">
@@ -1456,311 +1471,311 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="8"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="8"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="8"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="8"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="8"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="8"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="8"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="8"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="8"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="8"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="8"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F16" s="8"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F17" s="8"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="8"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F19" s="8"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F20" s="8"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F21" s="8"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F21" s="10"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E21">
@@ -1793,69 +1808,69 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="11" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>